<commit_message>
Before adding interpolation for GR projection
</commit_message>
<xml_diff>
--- a/et_custom_input_data.xlsx
+++ b/et_custom_input_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\kyleswartz\projects\ETtoKGT\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2ACB2895-257D-4B24-87B8-0AA76F425200}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B474354C-AF7A-4285-A46A-6BD9654C5A54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{D50FBC2E-9E0F-4B27-B5AE-2B4706E55574}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="160">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="160">
   <si>
     <t>Unnamed: 0</t>
   </si>
@@ -930,7 +930,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7095CECD-B3C1-479B-A395-9B195FCE92D6}">
-  <dimension ref="A1:ES8"/>
+  <dimension ref="A1:ES11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="20" max="20" width="8.88671875" style="4"/>
@@ -3719,6 +3719,1353 @@
         <v>136.9653878</v>
       </c>
     </row>
+    <row r="9" spans="1:149" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>0</v>
+      </c>
+      <c r="B9" t="s">
+        <v>149</v>
+      </c>
+      <c r="C9">
+        <v>0.48</v>
+      </c>
+      <c r="D9">
+        <v>0</v>
+      </c>
+      <c r="E9">
+        <v>0</v>
+      </c>
+      <c r="F9">
+        <v>0.48</v>
+      </c>
+      <c r="G9">
+        <v>0.02</v>
+      </c>
+      <c r="H9">
+        <v>0.02</v>
+      </c>
+      <c r="I9">
+        <v>0</v>
+      </c>
+      <c r="J9">
+        <v>1</v>
+      </c>
+      <c r="K9">
+        <v>3454.8464669999998</v>
+      </c>
+      <c r="L9">
+        <v>15296.24612</v>
+      </c>
+      <c r="M9">
+        <v>19370.285759999999</v>
+      </c>
+      <c r="N9">
+        <v>23.749503539999999</v>
+      </c>
+      <c r="O9">
+        <v>10.71769387</v>
+      </c>
+      <c r="P9">
+        <v>4.0400000000000003E-6</v>
+      </c>
+      <c r="Q9">
+        <v>6.1700000000000002E-6</v>
+      </c>
+      <c r="R9">
+        <v>251.61732309999999</v>
+      </c>
+      <c r="S9">
+        <v>180.586792</v>
+      </c>
+      <c r="T9" s="4">
+        <v>0.590243085</v>
+      </c>
+      <c r="U9">
+        <v>250</v>
+      </c>
+      <c r="V9">
+        <v>500</v>
+      </c>
+      <c r="W9" s="4">
+        <v>250</v>
+      </c>
+      <c r="X9" s="4">
+        <v>0.2</v>
+      </c>
+      <c r="Y9">
+        <v>500</v>
+      </c>
+      <c r="Z9">
+        <v>114.596</v>
+      </c>
+      <c r="AA9">
+        <v>4.8170000000000002</v>
+      </c>
+      <c r="AB9">
+        <v>96.084999999999994</v>
+      </c>
+      <c r="AC9">
+        <v>0.45542277199999998</v>
+      </c>
+      <c r="AD9">
+        <v>2.9943729999999998E-3</v>
+      </c>
+      <c r="AE9" t="s">
+        <v>150</v>
+      </c>
+      <c r="AF9">
+        <v>164</v>
+      </c>
+      <c r="AG9">
+        <v>52</v>
+      </c>
+      <c r="AH9">
+        <v>2000</v>
+      </c>
+      <c r="AI9">
+        <v>16.931000000000001</v>
+      </c>
+      <c r="AJ9">
+        <v>180.58799999999999</v>
+      </c>
+      <c r="AK9">
+        <v>3460.84</v>
+      </c>
+      <c r="AL9">
+        <v>5.48</v>
+      </c>
+      <c r="AM9">
+        <v>2.3149717509999999</v>
+      </c>
+      <c r="AN9">
+        <v>0.31119999999999998</v>
+      </c>
+      <c r="AO9">
+        <v>251.6</v>
+      </c>
+      <c r="AP9">
+        <v>108.6838316</v>
+      </c>
+      <c r="AQ9">
+        <v>285.01247999999998</v>
+      </c>
+      <c r="AR9">
+        <v>110.44</v>
+      </c>
+      <c r="AS9">
+        <v>384.57</v>
+      </c>
+      <c r="AT9">
+        <v>181.756</v>
+      </c>
+      <c r="AU9">
+        <v>103.72799999999999</v>
+      </c>
+      <c r="AV9">
+        <v>78.028000000000006</v>
+      </c>
+      <c r="AW9">
+        <v>1.0228879660000001</v>
+      </c>
+      <c r="AX9">
+        <v>6.1456499999999997E-4</v>
+      </c>
+      <c r="AY9">
+        <v>249.3606667</v>
+      </c>
+      <c r="AZ9">
+        <v>103.72799999999999</v>
+      </c>
+      <c r="BA9">
+        <v>1.9219999999999999</v>
+      </c>
+      <c r="BB9">
+        <v>143.96</v>
+      </c>
+      <c r="BC9">
+        <v>0.86109132799999999</v>
+      </c>
+      <c r="BD9">
+        <v>2.5713613999999999E-2</v>
+      </c>
+      <c r="BE9">
+        <v>4.8244129999999996E-3</v>
+      </c>
+      <c r="BF9">
+        <v>0.100737432</v>
+      </c>
+      <c r="BG9">
+        <v>2.1614299999999999E-4</v>
+      </c>
+      <c r="BH9">
+        <v>5.2086074000000003E-2</v>
+      </c>
+      <c r="BI9">
+        <v>0.453460048</v>
+      </c>
+      <c r="BJ9">
+        <v>2.4708790000000001E-2</v>
+      </c>
+      <c r="BK9">
+        <v>9.8234493000000006E-2</v>
+      </c>
+      <c r="BL9">
+        <v>0.22919963500000001</v>
+      </c>
+      <c r="BM9">
+        <v>1453.6841870000001</v>
+      </c>
+      <c r="BN9">
+        <v>0.476258615</v>
+      </c>
+      <c r="BO9">
+        <v>2.8367983109999999</v>
+      </c>
+      <c r="BP9">
+        <v>6.4197078000000005E-2</v>
+      </c>
+      <c r="BQ9">
+        <v>1382.2900990000001</v>
+      </c>
+      <c r="BR9">
+        <v>572.84799610000005</v>
+      </c>
+      <c r="BS9">
+        <v>1042.2361960000001</v>
+      </c>
+      <c r="BT9">
+        <v>468.82416499999999</v>
+      </c>
+      <c r="BU9">
+        <v>192.5912342</v>
+      </c>
+      <c r="BV9">
+        <v>208.91441850000001</v>
+      </c>
+      <c r="BW9">
+        <v>8.0015981E-2</v>
+      </c>
+      <c r="BX9">
+        <v>240.04794290000001</v>
+      </c>
+      <c r="BY9">
+        <v>223.431613</v>
+      </c>
+      <c r="BZ9" s="4">
+        <v>3454.8464669999998</v>
+      </c>
+      <c r="CA9">
+        <v>3358.7692830000001</v>
+      </c>
+      <c r="CB9">
+        <v>16.462475430000001</v>
+      </c>
+      <c r="CC9">
+        <v>46.271406540000001</v>
+      </c>
+      <c r="CD9">
+        <v>45.715451539999997</v>
+      </c>
+      <c r="CE9">
+        <v>2.1874442000000001E-2</v>
+      </c>
+      <c r="CF9" s="2">
+        <v>1.08381E-5</v>
+      </c>
+      <c r="CG9" s="2">
+        <v>1.10306E-6</v>
+      </c>
+      <c r="CH9">
+        <v>906572.58589999995</v>
+      </c>
+      <c r="CI9">
+        <v>15.296246119999999</v>
+      </c>
+      <c r="CJ9">
+        <v>45.438765080000003</v>
+      </c>
+      <c r="CK9" s="4">
+        <v>23.749503539999999</v>
+      </c>
+      <c r="CL9">
+        <v>4.2106142999999999E-2</v>
+      </c>
+      <c r="CM9" s="2">
+        <v>6.17082E-6</v>
+      </c>
+      <c r="CN9" s="2">
+        <v>2.7980799999999998E-6</v>
+      </c>
+      <c r="CO9">
+        <v>357388.13919999998</v>
+      </c>
+      <c r="CP9">
+        <v>18.03892072</v>
+      </c>
+      <c r="CQ9">
+        <v>24.73414</v>
+      </c>
+      <c r="CR9">
+        <v>48.265258959999997</v>
+      </c>
+      <c r="CS9">
+        <v>2.0718836000000001E-2</v>
+      </c>
+      <c r="CT9" s="2">
+        <v>1.95356E-5</v>
+      </c>
+      <c r="CU9" s="2">
+        <v>3.2153999999999999E-9</v>
+      </c>
+      <c r="CV9">
+        <v>311003330.30000001</v>
+      </c>
+      <c r="CW9">
+        <v>16.956278170000001</v>
+      </c>
+      <c r="CX9">
+        <v>33.403267239999998</v>
+      </c>
+      <c r="CY9">
+        <v>46.016555449999998</v>
+      </c>
+      <c r="CZ9">
+        <v>2.1731309000000001E-2</v>
+      </c>
+      <c r="DA9" s="2">
+        <v>1.46722E-5</v>
+      </c>
+      <c r="DB9" s="2">
+        <v>7.5787200000000005E-7</v>
+      </c>
+      <c r="DC9">
+        <v>1319484.453</v>
+      </c>
+      <c r="DD9">
+        <v>-7733.9118230000004</v>
+      </c>
+      <c r="DE9">
+        <v>-7733.9118230000004</v>
+      </c>
+      <c r="DF9">
+        <v>49.317869760000001</v>
+      </c>
+      <c r="DG9">
+        <v>18.03892072</v>
+      </c>
+      <c r="DH9">
+        <v>180.5926</v>
+      </c>
+      <c r="DI9" s="2">
+        <v>1.00113E-5</v>
+      </c>
+      <c r="DJ9">
+        <v>0.94</v>
+      </c>
+      <c r="DK9">
+        <v>0.94</v>
+      </c>
+      <c r="DL9">
+        <v>50781.434370000003</v>
+      </c>
+      <c r="DM9">
+        <v>50781.434370000003</v>
+      </c>
+      <c r="DN9">
+        <v>46.016555449999998</v>
+      </c>
+      <c r="DO9">
+        <v>16.956278170000001</v>
+      </c>
+      <c r="DP9">
+        <v>180.5926</v>
+      </c>
+      <c r="DQ9" s="2">
+        <v>1.0650500000000001E-5</v>
+      </c>
+      <c r="DR9">
+        <v>1</v>
+      </c>
+      <c r="DS9">
+        <v>1</v>
+      </c>
+      <c r="DT9">
+        <v>93128.501780000006</v>
+      </c>
+      <c r="DU9">
+        <v>93128.501780000006</v>
+      </c>
+      <c r="DV9">
+        <v>45.715752180000003</v>
+      </c>
+      <c r="DW9">
+        <v>16.462982400000001</v>
+      </c>
+      <c r="DX9">
+        <v>180.5926</v>
+      </c>
+      <c r="DY9" s="2">
+        <v>1.0969600000000001E-5</v>
+      </c>
+      <c r="DZ9">
+        <v>1</v>
+      </c>
+      <c r="EA9">
+        <v>1</v>
+      </c>
+      <c r="EB9">
+        <v>140812.95379999999</v>
+      </c>
+      <c r="EC9">
+        <v>140812.95379999999</v>
+      </c>
+      <c r="ED9">
+        <v>23.75028618</v>
+      </c>
+      <c r="EE9">
+        <v>9.2622520000000003E-3</v>
+      </c>
+      <c r="EF9" s="2">
+        <v>6.0556999999999999E-7</v>
+      </c>
+      <c r="EG9">
+        <v>15.295102</v>
+      </c>
+      <c r="EH9" s="2">
+        <v>1.1807199999999999E-5</v>
+      </c>
+      <c r="EI9">
+        <v>2.253734219</v>
+      </c>
+      <c r="EJ9">
+        <v>47.055460930000002</v>
+      </c>
+      <c r="EK9" s="4">
+        <v>260.56978149999998</v>
+      </c>
+      <c r="EL9">
+        <v>256.22807749999998</v>
+      </c>
+      <c r="EM9" s="4">
+        <v>18038.920719999998</v>
+      </c>
+      <c r="EN9">
+        <v>16462.475429999999</v>
+      </c>
+      <c r="EO9">
+        <v>15296.24612</v>
+      </c>
+      <c r="EP9" s="4">
+        <v>8.0000000000000007E-5</v>
+      </c>
+      <c r="EQ9" t="s">
+        <v>151</v>
+      </c>
+      <c r="ER9" s="4">
+        <v>251.6173225</v>
+      </c>
+      <c r="ES9">
+        <v>136.9653878</v>
+      </c>
+    </row>
+    <row r="10" spans="1:149" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>0</v>
+      </c>
+      <c r="B10" t="s">
+        <v>149</v>
+      </c>
+      <c r="C10">
+        <v>0.48</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+      <c r="E10">
+        <v>0</v>
+      </c>
+      <c r="F10">
+        <v>0.48</v>
+      </c>
+      <c r="G10">
+        <v>0.02</v>
+      </c>
+      <c r="H10">
+        <v>0.02</v>
+      </c>
+      <c r="I10">
+        <v>0</v>
+      </c>
+      <c r="J10">
+        <v>1</v>
+      </c>
+      <c r="K10">
+        <v>3454.8464669999998</v>
+      </c>
+      <c r="L10">
+        <v>15296.24612</v>
+      </c>
+      <c r="M10">
+        <v>19370.285759999999</v>
+      </c>
+      <c r="N10">
+        <v>23.749503539999999</v>
+      </c>
+      <c r="O10">
+        <v>10.71769387</v>
+      </c>
+      <c r="P10">
+        <v>4.0400000000000003E-6</v>
+      </c>
+      <c r="Q10">
+        <v>6.1700000000000002E-6</v>
+      </c>
+      <c r="R10">
+        <v>251.61732309999999</v>
+      </c>
+      <c r="S10">
+        <v>180.586792</v>
+      </c>
+      <c r="T10" s="4">
+        <v>0.590243085</v>
+      </c>
+      <c r="U10">
+        <v>250</v>
+      </c>
+      <c r="V10">
+        <v>500</v>
+      </c>
+      <c r="W10" s="4">
+        <v>275</v>
+      </c>
+      <c r="X10" s="4">
+        <v>1.65</v>
+      </c>
+      <c r="Y10">
+        <v>500</v>
+      </c>
+      <c r="Z10">
+        <v>114.596</v>
+      </c>
+      <c r="AA10">
+        <v>4.8170000000000002</v>
+      </c>
+      <c r="AB10">
+        <v>96.084999999999994</v>
+      </c>
+      <c r="AC10">
+        <v>0.45542277199999998</v>
+      </c>
+      <c r="AD10">
+        <v>2.9943729999999998E-3</v>
+      </c>
+      <c r="AE10" t="s">
+        <v>150</v>
+      </c>
+      <c r="AF10">
+        <v>164</v>
+      </c>
+      <c r="AG10">
+        <v>52</v>
+      </c>
+      <c r="AH10">
+        <v>2000</v>
+      </c>
+      <c r="AI10">
+        <v>16.931000000000001</v>
+      </c>
+      <c r="AJ10">
+        <v>180.58799999999999</v>
+      </c>
+      <c r="AK10">
+        <v>3460.84</v>
+      </c>
+      <c r="AL10">
+        <v>5.48</v>
+      </c>
+      <c r="AM10">
+        <v>2.3149717509999999</v>
+      </c>
+      <c r="AN10">
+        <v>0.31119999999999998</v>
+      </c>
+      <c r="AO10">
+        <v>251.6</v>
+      </c>
+      <c r="AP10">
+        <v>108.6838316</v>
+      </c>
+      <c r="AQ10">
+        <v>285.01247999999998</v>
+      </c>
+      <c r="AR10">
+        <v>110.44</v>
+      </c>
+      <c r="AS10">
+        <v>384.57</v>
+      </c>
+      <c r="AT10">
+        <v>181.756</v>
+      </c>
+      <c r="AU10">
+        <v>103.72799999999999</v>
+      </c>
+      <c r="AV10">
+        <v>78.028000000000006</v>
+      </c>
+      <c r="AW10">
+        <v>1.0228879660000001</v>
+      </c>
+      <c r="AX10">
+        <v>6.1456499999999997E-4</v>
+      </c>
+      <c r="AY10">
+        <v>249.3606667</v>
+      </c>
+      <c r="AZ10">
+        <v>103.72799999999999</v>
+      </c>
+      <c r="BA10">
+        <v>1.9219999999999999</v>
+      </c>
+      <c r="BB10">
+        <v>143.96</v>
+      </c>
+      <c r="BC10">
+        <v>0.86109132799999999</v>
+      </c>
+      <c r="BD10">
+        <v>2.5713613999999999E-2</v>
+      </c>
+      <c r="BE10">
+        <v>4.8244129999999996E-3</v>
+      </c>
+      <c r="BF10">
+        <v>0.100737432</v>
+      </c>
+      <c r="BG10">
+        <v>2.1614299999999999E-4</v>
+      </c>
+      <c r="BH10">
+        <v>5.2086074000000003E-2</v>
+      </c>
+      <c r="BI10">
+        <v>0.453460048</v>
+      </c>
+      <c r="BJ10">
+        <v>2.4708790000000001E-2</v>
+      </c>
+      <c r="BK10">
+        <v>9.8234493000000006E-2</v>
+      </c>
+      <c r="BL10">
+        <v>0.22919963500000001</v>
+      </c>
+      <c r="BM10">
+        <v>1453.6841870000001</v>
+      </c>
+      <c r="BN10">
+        <v>0.476258615</v>
+      </c>
+      <c r="BO10">
+        <v>2.8367983109999999</v>
+      </c>
+      <c r="BP10">
+        <v>6.4197078000000005E-2</v>
+      </c>
+      <c r="BQ10">
+        <v>1382.2900990000001</v>
+      </c>
+      <c r="BR10">
+        <v>572.84799610000005</v>
+      </c>
+      <c r="BS10">
+        <v>1042.2361960000001</v>
+      </c>
+      <c r="BT10">
+        <v>468.82416499999999</v>
+      </c>
+      <c r="BU10">
+        <v>192.5912342</v>
+      </c>
+      <c r="BV10">
+        <v>208.91441850000001</v>
+      </c>
+      <c r="BW10">
+        <v>8.0015981E-2</v>
+      </c>
+      <c r="BX10">
+        <v>240.04794290000001</v>
+      </c>
+      <c r="BY10">
+        <v>223.431613</v>
+      </c>
+      <c r="BZ10" s="4">
+        <v>3454.8464669999998</v>
+      </c>
+      <c r="CA10">
+        <v>3358.7692830000001</v>
+      </c>
+      <c r="CB10">
+        <v>16.462475430000001</v>
+      </c>
+      <c r="CC10">
+        <v>46.271406540000001</v>
+      </c>
+      <c r="CD10">
+        <v>45.715451539999997</v>
+      </c>
+      <c r="CE10">
+        <v>2.1874442000000001E-2</v>
+      </c>
+      <c r="CF10" s="2">
+        <v>1.08E-5</v>
+      </c>
+      <c r="CG10" s="2">
+        <v>1.1000000000000001E-6</v>
+      </c>
+      <c r="CH10">
+        <v>906572.58589999995</v>
+      </c>
+      <c r="CI10">
+        <v>15.296246119999999</v>
+      </c>
+      <c r="CJ10">
+        <v>45.438765080000003</v>
+      </c>
+      <c r="CK10" s="4">
+        <v>23.749503539999999</v>
+      </c>
+      <c r="CL10">
+        <v>4.2106142999999999E-2</v>
+      </c>
+      <c r="CM10" s="2">
+        <v>6.1700000000000002E-6</v>
+      </c>
+      <c r="CN10" s="2">
+        <v>2.7999999999999999E-6</v>
+      </c>
+      <c r="CO10">
+        <v>357388.13919999998</v>
+      </c>
+      <c r="CP10">
+        <v>18.03892072</v>
+      </c>
+      <c r="CQ10">
+        <v>24.73414</v>
+      </c>
+      <c r="CR10">
+        <v>48.265258959999997</v>
+      </c>
+      <c r="CS10">
+        <v>2.0718836000000001E-2</v>
+      </c>
+      <c r="CT10" s="2">
+        <v>1.95E-5</v>
+      </c>
+      <c r="CU10" s="2">
+        <v>3.22E-9</v>
+      </c>
+      <c r="CV10">
+        <v>311003330.30000001</v>
+      </c>
+      <c r="CW10">
+        <v>16.956278170000001</v>
+      </c>
+      <c r="CX10">
+        <v>33.403267239999998</v>
+      </c>
+      <c r="CY10">
+        <v>46.016555449999998</v>
+      </c>
+      <c r="CZ10">
+        <v>2.1731309000000001E-2</v>
+      </c>
+      <c r="DA10" s="2">
+        <v>1.47E-5</v>
+      </c>
+      <c r="DB10" s="2">
+        <v>7.5799999999999998E-7</v>
+      </c>
+      <c r="DC10">
+        <v>1319484.453</v>
+      </c>
+      <c r="DD10">
+        <v>-7733.9118230000004</v>
+      </c>
+      <c r="DE10">
+        <v>-7733.9118230000004</v>
+      </c>
+      <c r="DF10">
+        <v>49.317869760000001</v>
+      </c>
+      <c r="DG10">
+        <v>18.03892072</v>
+      </c>
+      <c r="DH10">
+        <v>180.5926</v>
+      </c>
+      <c r="DI10" s="2">
+        <v>1.0000000000000001E-5</v>
+      </c>
+      <c r="DJ10">
+        <v>0.94</v>
+      </c>
+      <c r="DK10">
+        <v>0.94</v>
+      </c>
+      <c r="DL10">
+        <v>50781.434370000003</v>
+      </c>
+      <c r="DM10">
+        <v>50781.434370000003</v>
+      </c>
+      <c r="DN10">
+        <v>46.016555449999998</v>
+      </c>
+      <c r="DO10">
+        <v>16.956278170000001</v>
+      </c>
+      <c r="DP10">
+        <v>180.5926</v>
+      </c>
+      <c r="DQ10" s="2">
+        <v>1.0699999999999999E-5</v>
+      </c>
+      <c r="DR10">
+        <v>1</v>
+      </c>
+      <c r="DS10">
+        <v>1</v>
+      </c>
+      <c r="DT10">
+        <v>93128.501780000006</v>
+      </c>
+      <c r="DU10">
+        <v>93128.501780000006</v>
+      </c>
+      <c r="DV10">
+        <v>45.715752180000003</v>
+      </c>
+      <c r="DW10">
+        <v>16.462982400000001</v>
+      </c>
+      <c r="DX10">
+        <v>180.5926</v>
+      </c>
+      <c r="DY10" s="2">
+        <v>1.1E-5</v>
+      </c>
+      <c r="DZ10">
+        <v>1</v>
+      </c>
+      <c r="EA10">
+        <v>1</v>
+      </c>
+      <c r="EB10">
+        <v>140812.95379999999</v>
+      </c>
+      <c r="EC10">
+        <v>140812.95379999999</v>
+      </c>
+      <c r="ED10">
+        <v>23.75028618</v>
+      </c>
+      <c r="EE10">
+        <v>9.2622520000000003E-3</v>
+      </c>
+      <c r="EF10" s="2">
+        <v>6.06E-7</v>
+      </c>
+      <c r="EG10">
+        <v>15.295102</v>
+      </c>
+      <c r="EH10" s="2">
+        <v>1.1800000000000001E-5</v>
+      </c>
+      <c r="EI10">
+        <v>2.253734219</v>
+      </c>
+      <c r="EJ10">
+        <v>47.055460930000002</v>
+      </c>
+      <c r="EK10" s="4">
+        <v>260.56978149999998</v>
+      </c>
+      <c r="EL10">
+        <v>256.22807749999998</v>
+      </c>
+      <c r="EM10" s="4">
+        <v>18038.920719999998</v>
+      </c>
+      <c r="EN10">
+        <v>16462.475429999999</v>
+      </c>
+      <c r="EO10">
+        <v>15296.24612</v>
+      </c>
+      <c r="EP10" s="4">
+        <v>8.0000000000000007E-5</v>
+      </c>
+      <c r="EQ10" t="s">
+        <v>151</v>
+      </c>
+      <c r="ER10" s="4">
+        <v>251.6173225</v>
+      </c>
+      <c r="ES10">
+        <v>136.9653878</v>
+      </c>
+    </row>
+    <row r="11" spans="1:149" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>0</v>
+      </c>
+      <c r="B11" t="s">
+        <v>149</v>
+      </c>
+      <c r="C11">
+        <v>0.48</v>
+      </c>
+      <c r="D11">
+        <v>0</v>
+      </c>
+      <c r="E11">
+        <v>0</v>
+      </c>
+      <c r="F11">
+        <v>0.48</v>
+      </c>
+      <c r="G11">
+        <v>0.02</v>
+      </c>
+      <c r="H11">
+        <v>0.02</v>
+      </c>
+      <c r="I11">
+        <v>0</v>
+      </c>
+      <c r="J11">
+        <v>1</v>
+      </c>
+      <c r="K11">
+        <v>3454.8464669999998</v>
+      </c>
+      <c r="L11">
+        <v>15296.24612</v>
+      </c>
+      <c r="M11">
+        <v>19370.285759999999</v>
+      </c>
+      <c r="N11">
+        <v>23.749503539999999</v>
+      </c>
+      <c r="O11">
+        <v>10.71769387</v>
+      </c>
+      <c r="P11">
+        <v>4.0400000000000003E-6</v>
+      </c>
+      <c r="Q11">
+        <v>6.1700000000000002E-6</v>
+      </c>
+      <c r="R11">
+        <v>251.61732309999999</v>
+      </c>
+      <c r="S11">
+        <v>180.586792</v>
+      </c>
+      <c r="T11" s="4">
+        <v>0.590243085</v>
+      </c>
+      <c r="U11">
+        <v>250</v>
+      </c>
+      <c r="V11">
+        <v>500</v>
+      </c>
+      <c r="W11" s="4">
+        <v>250</v>
+      </c>
+      <c r="X11" s="4">
+        <v>0.5</v>
+      </c>
+      <c r="Y11">
+        <v>500</v>
+      </c>
+      <c r="Z11">
+        <v>114.596</v>
+      </c>
+      <c r="AA11">
+        <v>4.8170000000000002</v>
+      </c>
+      <c r="AB11">
+        <v>96.084999999999994</v>
+      </c>
+      <c r="AC11">
+        <v>0.45542277199999998</v>
+      </c>
+      <c r="AD11">
+        <v>2.9943729999999998E-3</v>
+      </c>
+      <c r="AE11" t="s">
+        <v>150</v>
+      </c>
+      <c r="AF11">
+        <v>164</v>
+      </c>
+      <c r="AG11">
+        <v>52</v>
+      </c>
+      <c r="AH11">
+        <v>2000</v>
+      </c>
+      <c r="AI11">
+        <v>16.931000000000001</v>
+      </c>
+      <c r="AJ11">
+        <v>180.58799999999999</v>
+      </c>
+      <c r="AK11">
+        <v>3460.84</v>
+      </c>
+      <c r="AL11">
+        <v>5.48</v>
+      </c>
+      <c r="AM11">
+        <v>2.3149717509999999</v>
+      </c>
+      <c r="AN11">
+        <v>0.31119999999999998</v>
+      </c>
+      <c r="AO11">
+        <v>251.6</v>
+      </c>
+      <c r="AP11">
+        <v>108.6838316</v>
+      </c>
+      <c r="AQ11">
+        <v>285.01247999999998</v>
+      </c>
+      <c r="AR11">
+        <v>110.44</v>
+      </c>
+      <c r="AS11">
+        <v>384.57</v>
+      </c>
+      <c r="AT11">
+        <v>181.756</v>
+      </c>
+      <c r="AU11">
+        <v>103.72799999999999</v>
+      </c>
+      <c r="AV11">
+        <v>78.028000000000006</v>
+      </c>
+      <c r="AW11">
+        <v>1.0228879660000001</v>
+      </c>
+      <c r="AX11">
+        <v>6.1456499999999997E-4</v>
+      </c>
+      <c r="AY11">
+        <v>249.3606667</v>
+      </c>
+      <c r="AZ11">
+        <v>103.72799999999999</v>
+      </c>
+      <c r="BA11">
+        <v>1.9219999999999999</v>
+      </c>
+      <c r="BB11">
+        <v>143.96</v>
+      </c>
+      <c r="BC11">
+        <v>0.86109132799999999</v>
+      </c>
+      <c r="BD11">
+        <v>2.5713613999999999E-2</v>
+      </c>
+      <c r="BE11">
+        <v>4.8244129999999996E-3</v>
+      </c>
+      <c r="BF11">
+        <v>0.100737432</v>
+      </c>
+      <c r="BG11">
+        <v>2.1614299999999999E-4</v>
+      </c>
+      <c r="BH11">
+        <v>5.2086074000000003E-2</v>
+      </c>
+      <c r="BI11">
+        <v>0.453460048</v>
+      </c>
+      <c r="BJ11">
+        <v>2.4708790000000001E-2</v>
+      </c>
+      <c r="BK11">
+        <v>9.8234493000000006E-2</v>
+      </c>
+      <c r="BL11">
+        <v>0.22919963500000001</v>
+      </c>
+      <c r="BM11">
+        <v>1453.6841870000001</v>
+      </c>
+      <c r="BN11">
+        <v>0.476258615</v>
+      </c>
+      <c r="BO11">
+        <v>2.8367983109999999</v>
+      </c>
+      <c r="BP11">
+        <v>6.4197078000000005E-2</v>
+      </c>
+      <c r="BQ11">
+        <v>1382.2900990000001</v>
+      </c>
+      <c r="BR11">
+        <v>572.84799610000005</v>
+      </c>
+      <c r="BS11">
+        <v>1042.2361960000001</v>
+      </c>
+      <c r="BT11">
+        <v>468.82416499999999</v>
+      </c>
+      <c r="BU11">
+        <v>192.5912342</v>
+      </c>
+      <c r="BV11">
+        <v>208.91441850000001</v>
+      </c>
+      <c r="BW11">
+        <v>8.0015981E-2</v>
+      </c>
+      <c r="BX11">
+        <v>240.04794290000001</v>
+      </c>
+      <c r="BY11">
+        <v>223.431613</v>
+      </c>
+      <c r="BZ11" s="4">
+        <v>3454.8464669999998</v>
+      </c>
+      <c r="CA11">
+        <v>3358.7692830000001</v>
+      </c>
+      <c r="CB11">
+        <v>16.462475430000001</v>
+      </c>
+      <c r="CC11">
+        <v>46.271406540000001</v>
+      </c>
+      <c r="CD11">
+        <v>45.715451539999997</v>
+      </c>
+      <c r="CE11">
+        <v>2.1874442000000001E-2</v>
+      </c>
+      <c r="CF11" s="2">
+        <v>1.08E-5</v>
+      </c>
+      <c r="CG11" s="2">
+        <v>1.1000000000000001E-6</v>
+      </c>
+      <c r="CH11">
+        <v>906572.58589999995</v>
+      </c>
+      <c r="CI11">
+        <v>15.296246119999999</v>
+      </c>
+      <c r="CJ11">
+        <v>45.438765080000003</v>
+      </c>
+      <c r="CK11" s="4">
+        <v>23.749503539999999</v>
+      </c>
+      <c r="CL11">
+        <v>4.2106142999999999E-2</v>
+      </c>
+      <c r="CM11" s="2">
+        <v>6.1700000000000002E-6</v>
+      </c>
+      <c r="CN11" s="2">
+        <v>2.7999999999999999E-6</v>
+      </c>
+      <c r="CO11">
+        <v>357388.13919999998</v>
+      </c>
+      <c r="CP11">
+        <v>18.03892072</v>
+      </c>
+      <c r="CQ11">
+        <v>24.73414</v>
+      </c>
+      <c r="CR11">
+        <v>48.265258959999997</v>
+      </c>
+      <c r="CS11">
+        <v>2.0718836000000001E-2</v>
+      </c>
+      <c r="CT11" s="2">
+        <v>1.95E-5</v>
+      </c>
+      <c r="CU11" s="2">
+        <v>3.22E-9</v>
+      </c>
+      <c r="CV11">
+        <v>311003330.30000001</v>
+      </c>
+      <c r="CW11">
+        <v>16.956278170000001</v>
+      </c>
+      <c r="CX11">
+        <v>33.403267239999998</v>
+      </c>
+      <c r="CY11">
+        <v>46.016555449999998</v>
+      </c>
+      <c r="CZ11">
+        <v>2.1731309000000001E-2</v>
+      </c>
+      <c r="DA11" s="2">
+        <v>1.47E-5</v>
+      </c>
+      <c r="DB11" s="2">
+        <v>7.5799999999999998E-7</v>
+      </c>
+      <c r="DC11">
+        <v>1319484.453</v>
+      </c>
+      <c r="DD11">
+        <v>-7733.9118230000004</v>
+      </c>
+      <c r="DE11">
+        <v>-7733.9118230000004</v>
+      </c>
+      <c r="DF11">
+        <v>49.317869760000001</v>
+      </c>
+      <c r="DG11">
+        <v>18.03892072</v>
+      </c>
+      <c r="DH11">
+        <v>180.5926</v>
+      </c>
+      <c r="DI11" s="2">
+        <v>1.0000000000000001E-5</v>
+      </c>
+      <c r="DJ11">
+        <v>0.94</v>
+      </c>
+      <c r="DK11">
+        <v>0.94</v>
+      </c>
+      <c r="DL11">
+        <v>50781.434370000003</v>
+      </c>
+      <c r="DM11">
+        <v>50781.434370000003</v>
+      </c>
+      <c r="DN11">
+        <v>46.016555449999998</v>
+      </c>
+      <c r="DO11">
+        <v>16.956278170000001</v>
+      </c>
+      <c r="DP11">
+        <v>180.5926</v>
+      </c>
+      <c r="DQ11" s="2">
+        <v>1.0699999999999999E-5</v>
+      </c>
+      <c r="DR11">
+        <v>1</v>
+      </c>
+      <c r="DS11">
+        <v>1</v>
+      </c>
+      <c r="DT11">
+        <v>93128.501780000006</v>
+      </c>
+      <c r="DU11">
+        <v>93128.501780000006</v>
+      </c>
+      <c r="DV11">
+        <v>45.715752180000003</v>
+      </c>
+      <c r="DW11">
+        <v>16.462982400000001</v>
+      </c>
+      <c r="DX11">
+        <v>180.5926</v>
+      </c>
+      <c r="DY11" s="2">
+        <v>1.1E-5</v>
+      </c>
+      <c r="DZ11">
+        <v>1</v>
+      </c>
+      <c r="EA11">
+        <v>1</v>
+      </c>
+      <c r="EB11">
+        <v>140812.95379999999</v>
+      </c>
+      <c r="EC11">
+        <v>140812.95379999999</v>
+      </c>
+      <c r="ED11">
+        <v>23.75028618</v>
+      </c>
+      <c r="EE11">
+        <v>9.2622520000000003E-3</v>
+      </c>
+      <c r="EF11" s="2">
+        <v>6.06E-7</v>
+      </c>
+      <c r="EG11">
+        <v>15.295102</v>
+      </c>
+      <c r="EH11" s="2">
+        <v>1.1800000000000001E-5</v>
+      </c>
+      <c r="EI11">
+        <v>2.253734219</v>
+      </c>
+      <c r="EJ11">
+        <v>47.055460930000002</v>
+      </c>
+      <c r="EK11" s="4">
+        <v>260.56978149999998</v>
+      </c>
+      <c r="EL11">
+        <v>256.22807749999998</v>
+      </c>
+      <c r="EM11" s="4">
+        <v>18038.920719999998</v>
+      </c>
+      <c r="EN11">
+        <v>16462.475429999999</v>
+      </c>
+      <c r="EO11">
+        <v>15296.24612</v>
+      </c>
+      <c r="EP11" s="4">
+        <v>8.0000000000000007E-5</v>
+      </c>
+      <c r="EQ11" t="s">
+        <v>151</v>
+      </c>
+      <c r="ER11" s="4">
+        <v>260.56978149999998</v>
+      </c>
+      <c r="ES11">
+        <v>136.9653878</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>

</xml_diff>